<commit_message>
Add broker-ready execution mode settings
</commit_message>
<xml_diff>
--- a/reports/quant_strategy_research_report.xlsx
+++ b/reports/quant_strategy_research_report.xlsx
@@ -530,7 +530,7 @@
         <v>-7.88</v>
       </c>
       <c r="L2" t="n">
-        <v>12401.25</v>
+        <v>12401.24</v>
       </c>
       <c r="M2" t="n">
         <v>19</v>
@@ -626,7 +626,7 @@
         <v>-10.98</v>
       </c>
       <c r="L4" t="n">
-        <v>13550.63</v>
+        <v>13550.62</v>
       </c>
       <c r="M4" t="n">
         <v>16</v>
@@ -722,7 +722,7 @@
         <v>-8.9</v>
       </c>
       <c r="L6" t="n">
-        <v>13738.27</v>
+        <v>13738.28</v>
       </c>
       <c r="M6" t="n">
         <v>23</v>
@@ -770,7 +770,7 @@
         <v>-10.37</v>
       </c>
       <c r="L7" t="n">
-        <v>14618.87</v>
+        <v>14618.86</v>
       </c>
       <c r="M7" t="n">
         <v>15</v>
@@ -818,7 +818,7 @@
         <v>-11.53</v>
       </c>
       <c r="L8" t="n">
-        <v>16548.4</v>
+        <v>16548.39</v>
       </c>
       <c r="M8" t="n">
         <v>9</v>
@@ -866,7 +866,7 @@
         <v>-11.53</v>
       </c>
       <c r="L9" t="n">
-        <v>15883.47</v>
+        <v>15883.45</v>
       </c>
       <c r="M9" t="n">
         <v>11</v>
@@ -914,7 +914,7 @@
         <v>-14.88</v>
       </c>
       <c r="L10" t="n">
-        <v>16879.99</v>
+        <v>16879.98</v>
       </c>
       <c r="M10" t="n">
         <v>23</v>
@@ -962,7 +962,7 @@
         <v>-16.53</v>
       </c>
       <c r="L11" t="n">
-        <v>16361.73</v>
+        <v>16361.72</v>
       </c>
       <c r="M11" t="n">
         <v>20</v>
@@ -1576,7 +1576,7 @@
         <v>-11.53</v>
       </c>
       <c r="L2" t="n">
-        <v>16548.4</v>
+        <v>16548.39</v>
       </c>
       <c r="M2" t="n">
         <v>9</v>
@@ -1624,7 +1624,7 @@
         <v>-11.53</v>
       </c>
       <c r="L3" t="n">
-        <v>15883.47</v>
+        <v>15883.45</v>
       </c>
       <c r="M3" t="n">
         <v>11</v>
@@ -1672,7 +1672,7 @@
         <v>-14.88</v>
       </c>
       <c r="L4" t="n">
-        <v>16879.99</v>
+        <v>16879.98</v>
       </c>
       <c r="M4" t="n">
         <v>23</v>
@@ -2094,7 +2094,7 @@
         <v>-14.88</v>
       </c>
       <c r="L6" t="n">
-        <v>16879.99</v>
+        <v>16879.98</v>
       </c>
       <c r="M6" t="n">
         <v>23</v>
@@ -2228,7 +2228,7 @@
         <v>-7.88</v>
       </c>
       <c r="L2" t="n">
-        <v>12401.25</v>
+        <v>12401.24</v>
       </c>
       <c r="M2" t="n">
         <v>19</v>
@@ -2276,7 +2276,7 @@
         <v>-8.9</v>
       </c>
       <c r="L3" t="n">
-        <v>13738.27</v>
+        <v>13738.28</v>
       </c>
       <c r="M3" t="n">
         <v>23</v>
@@ -2372,7 +2372,7 @@
         <v>-10.37</v>
       </c>
       <c r="L5" t="n">
-        <v>14618.87</v>
+        <v>14618.86</v>
       </c>
       <c r="M5" t="n">
         <v>15</v>
@@ -2420,7 +2420,7 @@
         <v>-10.98</v>
       </c>
       <c r="L6" t="n">
-        <v>13550.63</v>
+        <v>13550.62</v>
       </c>
       <c r="M6" t="n">
         <v>16</v>

</xml_diff>